<commit_message>
Decrease font size of PI address from 12 to 11
</commit_message>
<xml_diff>
--- a/web/templates/pi/PI-template.xlsx
+++ b/web/templates/pi/PI-template.xlsx
@@ -249,7 +249,7 @@
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* (#,##0);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="_ * #,##0.00_ ;_ * -#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="37" x14ac:knownFonts="1">
+  <fonts count="38" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -283,6 +283,19 @@
       <color theme="1"/>
       <sz val="12"/>
       <name val="Times New Roman"/>
+    </font>
+    <font>
+      <charset val="134"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
+      <charset val="134"/>
+      <color theme="1"/>
+      <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <u/>
@@ -332,12 +345,6 @@
       <charset val="134"/>
       <color theme="1"/>
       <sz val="10"/>
-      <name val="Times New Roman"/>
-    </font>
-    <font>
-      <charset val="134"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <name val="Times New Roman"/>
     </font>
     <font>
@@ -866,226 +873,226 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="4" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="18" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="23" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="14" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="26" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="4" fontId="26" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="27" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="28" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="29" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="22" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="12" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="25" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="4" fontId="25" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="26" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="27" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="28" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="28" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="12" fillId="6" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="28" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="28" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="29" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="29" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="29" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="14" fillId="6" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="29" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="29" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="30" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="30" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="31" fillId="3" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="32" fillId="3" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="32" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="33" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="31" fillId="3" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="10" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="32" fillId="3" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="33" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="34" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="34" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="34" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="32" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="35" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="35" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="33" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1097,13 +1104,13 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1115,100 +1122,100 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="31" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="32" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="35" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="36" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="35" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="36" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="35" fillId="9" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="36" fillId="9" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="9" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="9" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="35" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="36" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="35" fillId="10" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="36" fillId="10" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="10" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="10" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="36" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="36" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="11" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="18" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="26" fillId="3" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="27" fillId="3" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>

</xml_diff>